<commit_message>
Add update log and summer release notes
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R22ea46d57f6d4d15"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Ra4ab3ec8cb164712"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R41f8d7cefdc549b1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R4a43eeee9d2e4d34"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -54158,7 +54158,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R2bec449f23244dc9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7eab4003e30449d9"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54335,7 +54335,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>151a2d7e08baa95e13e124a3af98d44957d7605acd6523dc60335990866e7472</x:v>
+        <x:v>74fdd36df75125f8e1fcf2d2053d1eea0dff35eb34ea710193cb7e255b340544</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -54343,7 +54343,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>a2f3814677bb5fbda2b44ace7a25b752e88f750df49e081cb72dea2bd8bcb353</x:v>
+        <x:v>70241989a5d288b0e53ebd9d904c6fb9e7b496fefa34214aafe1efc3540a93f7</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>

<commit_message>
Complete recent work analysis update history
</commit_message>
<xml_diff>
--- a/data/yuri_classification_database_comparison.xlsx
+++ b/data/yuri_classification_database_comparison.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R41f8d7cefdc549b1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="R4a43eeee9d2e4d34"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="数据库标签对照" sheetId="1" r:id="R5132cce5942f4908"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="说明与来源" sheetId="2" r:id="Rebb22c770a944cd6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -54158,7 +54158,7 @@
   </x:conditionalFormatting>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R7eab4003e30449d9"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rbf586e0fc8dd47bd"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -54335,7 +54335,7 @@
         <x:v>数据库源 SHA-256</x:v>
       </x:c>
       <x:c r="B23" s="27" t="str">
-        <x:v>74fdd36df75125f8e1fcf2d2053d1eea0dff35eb34ea710193cb7e255b340544</x:v>
+        <x:v>408851f843d65cb19fe72a52821e579b0f233bc466330a99fd334a7130a4c21b</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="31.5" customHeight="1">
@@ -54343,7 +54343,7 @@
         <x:v>发布计划 SHA-256</x:v>
       </x:c>
       <x:c r="B24" s="27" t="str">
-        <x:v>70241989a5d288b0e53ebd9d904c6fb9e7b496fefa34214aafe1efc3540a93f7</x:v>
+        <x:v>85a435915292f6d1277347121e382e691190e8de656f38361ca1a8c763f19f32</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="31.5" customHeight="1">

</xml_diff>